<commit_message>
added normalize values from load .xlsx files and increased size of files to 10mb
</commit_message>
<xml_diff>
--- a/data/Unit Of Measure catalog.xlsx
+++ b/data/Unit Of Measure catalog.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Profiles\iromo\Desktop\Propio\Validarores de txts\Enviar\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eoncr\OneDrive\Documentos\github_2026\DANA-API-WRITING\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86A9E867-6630-4805-9996-3A08A34E4A8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DF07C33-FCB5-45EC-B577-087DE1DF4523}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-107" yWindow="-107" windowWidth="20847" windowHeight="11111" xr2:uid="{ACFB17C9-C326-4356-AAFB-8D337BF4DB04}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{ACFB17C9-C326-4356-AAFB-8D337BF4DB04}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="133">
   <si>
     <t>Code</t>
   </si>
@@ -432,13 +432,19 @@
   </si>
   <si>
     <t>Yes</t>
+  </si>
+  <si>
+    <t>OZ</t>
+  </si>
+  <si>
+    <t>ONZA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -448,6 +454,14 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -475,9 +489,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -496,7 +511,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -812,16 +827,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1DF7170-42BE-4870-8F82-A24225D7F339}">
-  <dimension ref="A1:D67"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:G70"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="7.59765625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="29.296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.69921875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.69921875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -835,7 +850,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -846,7 +861,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -857,7 +872,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -868,7 +883,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -879,7 +894,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>87</v>
       </c>
@@ -890,7 +905,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -901,7 +916,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -915,7 +930,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>15</v>
       </c>
@@ -929,7 +944,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>17</v>
       </c>
@@ -940,7 +955,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>89</v>
       </c>
@@ -951,7 +966,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>91</v>
       </c>
@@ -962,7 +977,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>19</v>
       </c>
@@ -973,7 +988,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>21</v>
       </c>
@@ -984,7 +999,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>23</v>
       </c>
@@ -995,7 +1010,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>25</v>
       </c>
@@ -1009,7 +1024,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>27</v>
       </c>
@@ -1023,7 +1038,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>29</v>
       </c>
@@ -1037,7 +1052,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>31</v>
       </c>
@@ -1051,7 +1066,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>93</v>
       </c>
@@ -1065,7 +1080,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>32</v>
       </c>
@@ -1079,7 +1094,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>34</v>
       </c>
@@ -1093,7 +1108,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>36</v>
       </c>
@@ -1107,7 +1122,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>95</v>
       </c>
@@ -1118,7 +1133,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>38</v>
       </c>
@@ -1129,7 +1144,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>40</v>
       </c>
@@ -1143,7 +1158,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>97</v>
       </c>
@@ -1157,7 +1172,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>42</v>
       </c>
@@ -1168,7 +1183,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>44</v>
       </c>
@@ -1182,7 +1197,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>99</v>
       </c>
@@ -1196,7 +1211,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>101</v>
       </c>
@@ -1207,7 +1222,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>46</v>
       </c>
@@ -1221,7 +1236,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>48</v>
       </c>
@@ -1235,7 +1250,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>50</v>
       </c>
@@ -1246,7 +1261,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>52</v>
       </c>
@@ -1260,7 +1275,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>103</v>
       </c>
@@ -1271,7 +1286,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>105</v>
       </c>
@@ -1285,7 +1300,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>54</v>
       </c>
@@ -1299,7 +1314,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>56</v>
       </c>
@@ -1313,7 +1328,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>58</v>
       </c>
@@ -1327,7 +1342,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>60</v>
       </c>
@@ -1341,7 +1356,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>107</v>
       </c>
@@ -1352,7 +1367,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>109</v>
       </c>
@@ -1366,7 +1381,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>111</v>
       </c>
@@ -1380,7 +1395,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>113</v>
       </c>
@@ -1394,7 +1409,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>62</v>
       </c>
@@ -1405,7 +1420,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>64</v>
       </c>
@@ -1416,7 +1431,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>115</v>
       </c>
@@ -1427,7 +1442,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>117</v>
       </c>
@@ -1438,7 +1453,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>118</v>
       </c>
@@ -1449,7 +1464,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>119</v>
       </c>
@@ -1460,7 +1475,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>66</v>
       </c>
@@ -1471,7 +1486,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>68</v>
       </c>
@@ -1485,7 +1500,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>121</v>
       </c>
@@ -1496,7 +1511,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>70</v>
       </c>
@@ -1507,7 +1522,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>123</v>
       </c>
@@ -1518,7 +1533,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>125</v>
       </c>
@@ -1529,7 +1544,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>43</v>
       </c>
@@ -1540,7 +1555,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>127</v>
       </c>
@@ -1554,7 +1569,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>72</v>
       </c>
@@ -1568,7 +1583,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>74</v>
       </c>
@@ -1579,7 +1594,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>76</v>
       </c>
@@ -1593,7 +1608,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>78</v>
       </c>
@@ -1607,7 +1622,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>80</v>
       </c>
@@ -1621,7 +1636,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>82</v>
       </c>
@@ -1632,7 +1647,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>129</v>
       </c>
@@ -1646,7 +1661,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>84</v>
       </c>
@@ -1659,6 +1674,23 @@
       <c r="D67" t="s">
         <v>130</v>
       </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
+        <v>131</v>
+      </c>
+      <c r="B68" t="s">
+        <v>132</v>
+      </c>
+      <c r="C68" t="s">
+        <v>6</v>
+      </c>
+      <c r="D68" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G70" s="2"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:D67" xr:uid="{E1DF7170-42BE-4870-8F82-A24225D7F339}">
@@ -1671,23 +1703,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="44edee9e-58c3-4cb0-8794-845dc7881707" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101007E004D69D8F47542A6F75FC1BB7C545C" ma:contentTypeVersion="14" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="3e9c3c74e02bbfe88dcb30be42fd9cdc">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="dc4f5734-40cb-4add-bdd4-4883f1ee3b3d" xmlns:ns4="44edee9e-58c3-4cb0-8794-845dc7881707" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="22264fd6f16c5503d8873ee90f905871" ns3:_="" ns4:_="">
     <xsd:import namespace="dc4f5734-40cb-4add-bdd4-4883f1ee3b3d"/>
@@ -1912,32 +1927,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6648088B-8523-4F9A-9088-5DD3428EE29C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="44edee9e-58c3-4cb0-8794-845dc7881707"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="dc4f5734-40cb-4add-bdd4-4883f1ee3b3d"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E10FB31B-2FCF-4DFC-90D7-CF75F4958D74}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="44edee9e-58c3-4cb0-8794-845dc7881707" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{25AC1042-2317-4474-852F-B53FC45657B8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1954,4 +1961,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E10FB31B-2FCF-4DFC-90D7-CF75F4958D74}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6648088B-8523-4F9A-9088-5DD3428EE29C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="44edee9e-58c3-4cb0-8794-845dc7881707"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="dc4f5734-40cb-4add-bdd4-4883f1ee3b3d"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
new unit of measure added
</commit_message>
<xml_diff>
--- a/data/Unit Of Measure catalog.xlsx
+++ b/data/Unit Of Measure catalog.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eoncr\OneDrive\Documentos\github_2026\DANA-API-WRITING\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DF07C33-FCB5-45EC-B577-087DE1DF4523}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FD3F844-1C07-47E2-B75F-EA0CADF59671}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{ACFB17C9-C326-4356-AAFB-8D337BF4DB04}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$D$67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$D$68</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="134">
   <si>
     <t>Code</t>
   </si>
@@ -438,6 +438,9 @@
   </si>
   <si>
     <t>ONZA</t>
+  </si>
+  <si>
+    <t>P</t>
   </si>
 </sst>
 </file>
@@ -827,7 +830,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1DF7170-42BE-4870-8F82-A24225D7F339}">
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:G71"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="7.6328125" bestFit="1" customWidth="1"/>
@@ -1466,79 +1469,79 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>119</v>
+        <v>133</v>
       </c>
       <c r="B51" t="s">
         <v>120</v>
       </c>
       <c r="C51" t="s">
-        <v>86</v>
+        <v>6</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>66</v>
+        <v>119</v>
       </c>
       <c r="B52" t="s">
-        <v>67</v>
+        <v>120</v>
       </c>
       <c r="C52" t="s">
-        <v>6</v>
+        <v>86</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B53" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C53" t="s">
         <v>6</v>
-      </c>
-      <c r="D53" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>121</v>
+        <v>68</v>
       </c>
       <c r="B54" t="s">
-        <v>122</v>
+        <v>69</v>
       </c>
       <c r="C54" t="s">
-        <v>86</v>
+        <v>6</v>
+      </c>
+      <c r="D54" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>70</v>
+        <v>121</v>
       </c>
       <c r="B55" t="s">
-        <v>71</v>
+        <v>122</v>
       </c>
       <c r="C55" t="s">
-        <v>6</v>
+        <v>86</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>123</v>
+        <v>70</v>
       </c>
       <c r="B56" t="s">
-        <v>124</v>
+        <v>71</v>
       </c>
       <c r="C56" t="s">
-        <v>86</v>
+        <v>6</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B57" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C57" t="s">
         <v>86</v>
@@ -1546,10 +1549,10 @@
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>43</v>
+        <v>125</v>
       </c>
       <c r="B58" t="s">
-        <v>43</v>
+        <v>126</v>
       </c>
       <c r="C58" t="s">
         <v>86</v>
@@ -1557,27 +1560,24 @@
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>127</v>
+        <v>43</v>
       </c>
       <c r="B59" t="s">
-        <v>128</v>
+        <v>43</v>
       </c>
       <c r="C59" t="s">
         <v>86</v>
-      </c>
-      <c r="D59" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>72</v>
+        <v>127</v>
       </c>
       <c r="B60" t="s">
-        <v>73</v>
+        <v>128</v>
       </c>
       <c r="C60" t="s">
-        <v>6</v>
+        <v>86</v>
       </c>
       <c r="D60" t="s">
         <v>130</v>
@@ -1585,35 +1585,35 @@
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B61" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C61" t="s">
         <v>6</v>
+      </c>
+      <c r="D61" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B62" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C62" t="s">
         <v>6</v>
-      </c>
-      <c r="D62" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B63" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C63" t="s">
         <v>6</v>
@@ -1624,10 +1624,10 @@
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B64" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C64" t="s">
         <v>6</v>
@@ -1638,38 +1638,38 @@
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B65" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C65" t="s">
         <v>6</v>
+      </c>
+      <c r="D65" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>129</v>
+        <v>82</v>
       </c>
       <c r="B66" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C66" t="s">
-        <v>86</v>
-      </c>
-      <c r="D66" t="s">
-        <v>130</v>
+        <v>6</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>84</v>
+        <v>129</v>
       </c>
       <c r="B67" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="C67" t="s">
-        <v>6</v>
+        <v>86</v>
       </c>
       <c r="D67" t="s">
         <v>130</v>
@@ -1677,25 +1677,39 @@
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
+        <v>84</v>
+      </c>
+      <c r="B68" t="s">
+        <v>85</v>
+      </c>
+      <c r="C68" t="s">
+        <v>6</v>
+      </c>
+      <c r="D68" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
         <v>131</v>
       </c>
-      <c r="B68" t="s">
+      <c r="B69" t="s">
         <v>132</v>
       </c>
-      <c r="C68" t="s">
-        <v>6</v>
-      </c>
-      <c r="D68" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="G70" s="2"/>
+      <c r="C69" t="s">
+        <v>6</v>
+      </c>
+      <c r="D69" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G71" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D67" xr:uid="{E1DF7170-42BE-4870-8F82-A24225D7F339}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D67">
-      <sortCondition ref="A1:A67"/>
+  <autoFilter ref="A1:D68" xr:uid="{E1DF7170-42BE-4870-8F82-A24225D7F339}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D68">
+      <sortCondition ref="A1:A68"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1703,6 +1717,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101007E004D69D8F47542A6F75FC1BB7C545C" ma:contentTypeVersion="14" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="3e9c3c74e02bbfe88dcb30be42fd9cdc">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="dc4f5734-40cb-4add-bdd4-4883f1ee3b3d" xmlns:ns4="44edee9e-58c3-4cb0-8794-845dc7881707" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="22264fd6f16c5503d8873ee90f905871" ns3:_="" ns4:_="">
     <xsd:import namespace="dc4f5734-40cb-4add-bdd4-4883f1ee3b3d"/>
@@ -1927,15 +1950,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1945,6 +1959,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E10FB31B-2FCF-4DFC-90D7-CF75F4958D74}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{25AC1042-2317-4474-852F-B53FC45657B8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1959,14 +1981,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E10FB31B-2FCF-4DFC-90D7-CF75F4958D74}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>